<commit_message>
NICA: 4 reels corregidos al ángulo 'bloqueos que no dejan que el dinero llegue'; aviso de privacidad para el formulario de Meta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Fny2nKCcacyQTkz6nAHd2
</commit_message>
<xml_diff>
--- a/nica-apify/calendario/campana-live/campana-live-2026-10-29.xlsx
+++ b/nica-apify/calendario/campana-live/campana-live-2026-10-29.xlsx
@@ -660,36 +660,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>NO ES QUE NO SEPAS AHORRAR: TU CUERPO VIVE EL DINERO COMO PELIGRO</t>
+          <t>NO ES QUE TRABAJES POCO: TU CUERPO FRENA EL DINERO</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>No es que no sepas ahorrar. Es que tu cuerpo vive el dinero como un peligro.</t>
+          <t>No es que trabajes poco. Es que tu cuerpo vive el dinero como un peligro, y lo frena antes de que llegue.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>0:00–0:06 GANCHO: No es que no sepas ahorrar. Es que tu cuerpo vive el dinero como un peligro.
-0:06–0:13 GUARDAR: Guarda este video y compártelo con la amiga que siempre dice «a mí el dinero no me dura».
-0:13–0:22 DOLOR: Te pagan y en vez de paz sientes urgencia: gastar, pagar, que ya se vaya. No eres tú: es un programa de alarma.
-0:22–0:32 LISTA DE 3: Tres señales: uno, evitas ver tu cuenta del banco. Dos, gastas justo cuando estás estresada. Tres, cuando por fin te sobra algo, aparece una «emergencia».
-0:32–0:45 DATO: Los psicólogos Daniel Kahneman y Amos Tversky mostraron que perder nos duele más o menos el doble de lo que nos alegra ganar. Por eso tu cuerpo se pone en alerta con cada pago.
-0:45–0:51 [TU HISTORIA: cuándo te diste cuenta de que tu cuerpo se tensaba con el dinero]
-0:51–1:00 HACKEO (hazlo conmigo 3 veces): Mano en el pecho. Exhala largo. Repite conmigo: el dinero es seguro conmigo. El dinero es seguro conmigo. El dinero es seguro conmigo.
-1:00–1:08 REVELACIÓN: No es el dinero el que se va. Es tu cuerpo el que lo empuja para dejar de sentir peligro.
-1:08–1:21 CTA: El martes 3 de noviembre a las 11 de la mañana, hora CDMX, te guío gratis por Zoom en una hipnosis para hackear tus bloqueos con el dinero. Regístrate: el link está en mi perfil.</t>
+          <t>0:00–0:08 GANCHO: No es que trabajes poco. Es que tu cuerpo vive el dinero como un peligro, y lo frena antes de que llegue.
+0:08–0:16 GUARDAR: Guarda este video y compártelo con la amiga que siempre dice «trabajo y trabajo, y el dinero no se mueve».
+0:16–0:26 DOLOR: Te esfuerzas, haces todo, y el dinero no se mueve. Llega una oportunidad y algo en ti se tensa. No eres tú: es un programa de alarma.
+0:26–0:37 LISTA DE 3: Tres señales: uno, te da pena cobrar o decir tu precio. Dos, evitas ver tu cuenta del banco. Tres, cuando aparece una oportunidad, encuentras la razón para no tomarla.
+0:37–0:51 DATO: Los psicólogos Daniel Kahneman y Amos Tversky mostraron que perder nos duele más o menos el doble de lo que nos alegra ganar. Por eso tu cuerpo se pone en alerta cuando toca cobrar, pedir o arriesgar.
+0:51–0:57 [TU HISTORIA: cuándo te diste cuenta de que tu cuerpo se tensaba con el dinero]
+0:57–1:09 HACKEO (hazlo conmigo 3 veces): Mano en el pecho. Exhala largo. Repite conmigo: el dinero es seguro conmigo, me permito recibirlo. El dinero es seguro conmigo, me permito recibirlo. El dinero es seguro conmigo, me permito recibirlo.
+1:09–1:17 REVELACIÓN: No es que el dinero no quiera llegar. Es que tu cuerpo le cierra la puerta para dejar de sentir peligro.
+1:17–1:30 CTA: El martes 3 de noviembre a las 11 de la mañana, hora CDMX, te guío gratis por Zoom en una hipnosis para hackear tus bloqueos con el dinero. Regístrate: el link está en mi perfil.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>0–3 s: NO ES QUE NO SEPAS AHORRAR. Lista: 1 NO VES TU CUENTA · 2 GASTAS CON ESTRÉS · 3 LA «EMERGENCIA». Dato: Kahneman y Tversky. Final: «LIVE GRATIS · MARTES 3 NOV · 11 AM · LINK EN MI PERFIL».</t>
+          <t>0–3 s: NO ES QUE TRABAJES POCO. Lista: 1 PENA DE COBRAR · 2 NO VES TU CUENTA · 3 DEJAS PASAR OPORTUNIDADES. Dato: Kahneman y Tversky. Final: «LIVE GRATIS · MARTES 3 NOV · 11 AM · LINK EN MI PERFIL».</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>No es que no sepas ahorrar 💸 Tu cuerpo vive el dinero como peligro.
-El martes 3 de noviembre, 11 AM (CDMX), te guío gratis en una hipnosis para hackear ese programa. Regístrate: link en mi perfil 👆</t>
+          <t>No es que trabajes poco 💸 Tu cuerpo vive el dinero como peligro y lo frena antes de que llegue.
+El martes 3 de noviembre, 11 AM (CDMX), te guío gratis en una hipnosis para hackear ese bloqueo. Regístrate: link en mi perfil 👆</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -731,28 +731,28 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>CÓMO MANEJO EL DINERO CON UN CEREBRO TDAH</t>
+          <t>LO QUE ME FRENABA CON EL DINERO (TENGO TDAH)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Tengo TDAH y te voy a contar qué hago para que el dinero no se me vaya.</t>
+          <t>Tengo TDAH y te voy a contar qué me frenaba con el dinero, y qué hago hoy.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>[Cómo era tu relación con el dinero antes]
-[Una compra impulsiva que recuerdes]
-[Qué hackeo usas hoy antes de gastar]
+[Algo que te frenaba con el dinero: cobrar, pedir, decir tu precio… lo que tú hayas vivido]
+[Qué hackeo usas hoy]
 [Qué le dirías a otra mujer con TDAH]
-Cierre: ¿Tú eres de las que gasta para calmarse? Sin juicio, cuéntame.</t>
+Cierre: ¿Qué sientes que te frena a ti con el dinero? Sin juicio, cuéntame.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Dinero + TDAH 🧠💸 Lo que me funciona a mí, sin fórmulas mágicas.
-¿Tú gastas para calmarte? Cuéntame 👇</t>
+          <t>Dinero + TDAH 🧠 Lo que me frenaba y lo que me funciona hoy, sin fórmulas mágicas.
+¿Qué te frena a ti? Cuéntame 👇</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -794,35 +794,35 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>DI ESTO CUANDO TE PAGUEN LA QUINCENA</t>
+          <t>DÍA DE QUINCENA: DI ESTO PARA ABRIRTE A RECIBIR</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Hoy es quincena. Antes de pagar nada, di esto.</t>
+          <t>Hoy es quincena. Te haya llegado poco, mucho o nada, di esto.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>0:00–0:04 GANCHO: Hoy es quincena. Antes de pagar nada, di esto.
-0:04–0:10 GUARDAR: Guárdalo para cada quincena y compártelo con quien ya hizo cuentas y siente que no alcanza.
-0:10–0:19 DOLOR: Llega el dinero y en dos minutos ya lo repartiste en tu cabeza, con angustia. No eres tú: es el programa de «no alcanza».
-0:19–0:30 LISTA DE 3: Tres pasos: uno, pies en el piso y mano en el pecho. Dos, mira la cantidad completa, sin voltear la cara. Tres, di el decreto antes del primer pago.
-0:30–0:40 DATO: Una revisión de estudios de 2018, de Andrea Zaccaro, asoció la respiración lenta con más sensación de calma. Es una práctica de bienestar, no un tratamiento.
-0:40–0:44 [TU HISTORIA: cómo vivías tú la quincena antes]
-0:44–0:59 HACKEO (hazlo conmigo 3 veces): Exhala largo y repite conmigo: este dinero llega a mí y yo lo sostengo con calma. Este dinero llega a mí y yo lo sostengo con calma. Este dinero llega a mí y yo lo sostengo con calma.
-0:59–1:04 REVELACIÓN: La quincena no se va por pagar. Se va por pagar con miedo.
-1:04–1:17 CTA: El martes 3 de noviembre a las 11 de la mañana, hora CDMX, te guío gratis por Zoom en una hipnosis para hackear tus bloqueos con el dinero. Regístrate: el link está en mi perfil.</t>
+          <t>0:00–0:05 GANCHO: Hoy es quincena. Te haya llegado poco, mucho o nada, di esto.
+0:05–0:12 GUARDAR: Guárdalo para cada quincena y compártelo con quien trabaja mucho y siente que el dinero no se mueve.
+0:12–0:24 DOLOR: Ves que a otras les llega y a ti algo te frena: no pides, no cobras, no te atreves. No eres tú: es el programa de «el dinero no es para mí».
+0:24–0:36 LISTA DE 3: Tres pasos: uno, pies en el piso y mano en el pecho. Dos, di en voz alta la cantidad que te gustaría recibir, sin voltear la cara. Tres, di el decreto.
+0:36–0:46 DATO: Una revisión de estudios de 2018, de Andrea Zaccaro, asoció la respiración lenta con más sensación de calma. Es una práctica de bienestar, no un tratamiento.
+0:46–0:50 [TU HISTORIA: cómo vivías tú la quincena antes]
+0:50–1:02 HACKEO (hazlo conmigo 3 veces): Exhala largo y repite conmigo: me abro a recibir y lo sostengo con calma. Me abro a recibir y lo sostengo con calma. Me abro a recibir y lo sostengo con calma.
+1:02–1:09 REVELACIÓN: El dinero no se frena por falta de trabajo. Se frena cuando no te sientes segura de recibir.
+1:09–1:22 CTA: El martes 3 de noviembre a las 11 de la mañana, hora CDMX, te guío gratis por Zoom en una hipnosis para hackear tus bloqueos con el dinero. Regístrate: el link está en mi perfil.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>0–3 s: DI ESTO CUANDO TE PAGUEN LA QUINCENA. Pasos: 1 MANO EN EL PECHO · 2 MIRA LA CANTIDAD · 3 DECRETO. Final: «LIVE GRATIS · MARTES 3 NOV · 11 AM».</t>
+          <t>0–3 s: DÍA DE QUINCENA: DI ESTO. Pasos: 1 MANO EN EL PECHO · 2 DI LA CANTIDAD · 3 DECRETO. Final: «LIVE GRATIS · MARTES 3 NOV · 11 AM».</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Tu quincena merece otro estado 💰 Hazlo conmigo antes del primer pago.
+          <t>Llegue poco, mucho o nada esta quincena, di esto conmigo 💰 Ábrete a recibir.
 Y el martes 3 de noviembre, 11 AM (CDMX): hipnosis gratis para hackear tus bloqueos con el dinero. Link en mi perfil 👆</t>
         </is>
       </c>
@@ -865,35 +865,35 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>¿POR QUÉ SE TE VA LA QUINCENA EN 3 DÍAS?</t>
+          <t>¿POR QUÉ TRABAJAS TANTO Y EL DINERO NO SE MUEVE?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>¿Por qué la quincena te dura tres días aunque no compraste nada grande?</t>
+          <t>¿Por qué trabajas tanto y el dinero no se mueve?</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>0:00–0:05 GANCHO: ¿Por qué la quincena te dura tres días aunque no compraste nada grande?
-0:05–0:10 GUARDAR: Guarda este video y mándaselo a quien vive de quincena en quincena.
-0:10–0:16 DOLOR: No es que ganes poco ni que seas desordenada. Hay tres programas trabajando en automático.
-0:16–0:27 LISTA DE 3: Uno: compras para calmar el estrés, no porque lo necesites. Dos: no miras tu cuenta para no sentir miedo. Tres: repites lo que viste en casa con el dinero.
-0:27–0:36 DATO: Los economistas Karlsson, Loewenstein y Seppi lo llamaron «efecto avestruz»: evitamos mirar nuestra información de dinero cuando creemos que va a ser mala noticia.
-0:36–0:40 [TU HISTORIA: cuál de las 3 te pasaba a ti]
-0:40–0:49 HACKEO (hazlo conmigo 3 veces): Repite conmigo: miro mi dinero y lo dirijo yo. Miro mi dinero y lo dirijo yo. Miro mi dinero y lo dirijo yo.
-0:49–0:53 REVELACIÓN: Lo que no miras, lo maneja tu programa.
-0:53–1:06 CTA: El martes 3 de noviembre a las 11 de la mañana, hora CDMX, te guío gratis por Zoom en una hipnosis para hackear tus bloqueos con el dinero. Regístrate: el link está en mi perfil.</t>
+          <t>0:00–0:04 GANCHO: ¿Por qué trabajas tanto y el dinero no se mueve?
+0:04–0:09 GUARDAR: Guarda este video y mándaselo a quien trabaja el doble y sigue igual.
+0:09–0:17 DOLOR: No es flojera ni que no sepas hacerlo. Hay tres programas trabajando en automático que frenan el dinero antes de que llegue.
+0:17–0:30 LISTA DE 3: Uno: te da culpa cobrar, y cobras de menos o regalas tu trabajo. Dos: no miras tu cuenta para no sentir miedo. Tres: repites lo que oíste en casa, como «el dinero cuesta mucho trabajo».
+0:30–0:39 DATO: Los economistas Karlsson, Loewenstein y Seppi lo llamaron «efecto avestruz»: evitamos mirar nuestra información de dinero cuando creemos que va a ser mala noticia.
+0:39–0:43 [TU HISTORIA: cuál de las 3 te pasaba a ti]
+0:43–0:51 HACKEO (hazlo conmigo 3 veces): Repite conmigo: merezco recibir por lo que doy. Merezco recibir por lo que doy. Merezco recibir por lo que doy.
+0:51–0:55 REVELACIÓN: Lo que no miras, lo maneja tu programa.
+0:55–1:08 CTA: El martes 3 de noviembre a las 11 de la mañana, hora CDMX, te guío gratis por Zoom en una hipnosis para hackear tus bloqueos con el dinero. Regístrate: el link está en mi perfil.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>0–3 s: ¿POR QUÉ SE TE VA LA QUINCENA EN 3 DÍAS? Lista: 1 COMPRAS PARA CALMARTE · 2 NO MIRAS TU CUENTA · 3 REPITES LO DE CASA. Dato: efecto avestruz. Final: «LIVE GRATIS · MARTES 3 NOV · 11 AM».</t>
+          <t>0–3 s: ¿POR QUÉ TRABAJAS TANTO Y EL DINERO NO SE MUEVE? Lista: 1 CULPA AL COBRAR · 2 NO MIRAS TU CUENTA · 3 REPITES LO DE CASA. Dato: efecto avestruz. Final: «LIVE GRATIS · MARTES 3 NOV · 11 AM».</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>¿La quincena te dura 3 días? 🫠 No es mala suerte: son 3 programas.
+          <t>¿Trabajas tanto y el dinero no se mueve? 🫠 No es mala suerte: son 3 programas que lo frenan.
 Martes 3 de noviembre, 11 AM (CDMX): hipnosis gratis para hackearlos. Link en mi perfil 👆</t>
         </is>
       </c>

</xml_diff>